<commit_message>
feat(shipping): add per-day address overrides and integrate with shipping table
- Implemented per-day address override functionality in ShippingPage.
- Updated ShippingTable to utilize effective addresses based on overrides.
- Refactored CustomerOverlayTrigger to include permanent notes.
- Removed deprecated customer overlay trigger component.
- Enhanced address selection handling in AddressCell with persisting state.
- Updated related types and data handling for order day addresses.
- Removed unused orders data handling and types.
</commit_message>
<xml_diff>
--- a/data/test/addresses.xlsx
+++ b/data/test/addresses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,7 +454,7 @@
         <v>106.7033</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="3">
@@ -483,7 +483,7 @@
         <v>106.7071</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="4">
@@ -512,7 +512,7 @@
         <v>106.6981</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="5">
@@ -541,7 +541,7 @@
         <v>106.7009</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="6">
@@ -570,7 +570,7 @@
         <v>106.6961</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="7">
@@ -599,7 +599,7 @@
         <v>106.7012</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="8">
@@ -628,7 +628,7 @@
         <v>106.63</v>
       </c>
       <c r="I8" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="9">
@@ -657,7 +657,7 @@
         <v>106.6892</v>
       </c>
       <c r="I9" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="10">
@@ -686,7 +686,7 @@
         <v>106.6878</v>
       </c>
       <c r="I10" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="11">
@@ -715,7 +715,7 @@
         <v>106.693</v>
       </c>
       <c r="I11" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="12">
@@ -744,7 +744,7 @@
         <v>106.7052</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="13">
@@ -773,7 +773,7 @@
         <v>106.705</v>
       </c>
       <c r="I13" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="14">
@@ -802,7 +802,7 @@
         <v>106.7018</v>
       </c>
       <c r="I14" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="15">
@@ -831,7 +831,7 @@
         <v>106.6844</v>
       </c>
       <c r="I15" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="16">
@@ -860,7 +860,7 @@
         <v>106.684</v>
       </c>
       <c r="I16" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="17">
@@ -889,7 +889,7 @@
         <v>106.6803</v>
       </c>
       <c r="I17" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="18">
@@ -918,7 +918,7 @@
         <v>106.6411</v>
       </c>
       <c r="I18" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="19">
@@ -947,7 +947,7 @@
         <v>106.6762</v>
       </c>
       <c r="I19" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="20">
@@ -976,7 +976,7 @@
         <v>106.7098</v>
       </c>
       <c r="I20" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="21">
@@ -1005,7 +1005,7 @@
         <v>106.7122</v>
       </c>
       <c r="I21" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="22">
@@ -1034,7 +1034,7 @@
         <v>106.7199</v>
       </c>
       <c r="I22" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="23">
@@ -1063,7 +1063,7 @@
         <v>106.7221</v>
       </c>
       <c r="I23" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="24">
@@ -1092,7 +1092,7 @@
         <v>106.7</v>
       </c>
       <c r="I24" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="25">
@@ -1121,7 +1121,7 @@
         <v>106.7012</v>
       </c>
       <c r="I25" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="26">
@@ -1150,7 +1150,7 @@
         <v>106.71</v>
       </c>
       <c r="I26" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="27">
@@ -1179,7 +1179,7 @@
         <v>106.7071</v>
       </c>
       <c r="I27" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="28">
@@ -1208,7 +1208,7 @@
         <v>106.7033</v>
       </c>
       <c r="I28" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="29">
@@ -1237,7 +1237,7 @@
         <v>106.6905</v>
       </c>
       <c r="I29" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="30">
@@ -1266,7 +1266,7 @@
         <v>106.6522</v>
       </c>
       <c r="I30" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="31">
@@ -1295,7 +1295,7 @@
         <v>106.6478</v>
       </c>
       <c r="I31" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="32">
@@ -1324,7 +1324,7 @@
         <v>106.63</v>
       </c>
       <c r="I32" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="33">
@@ -1353,7 +1353,7 @@
         <v>106.7012</v>
       </c>
       <c r="I33" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="34">
@@ -1382,7 +1382,7 @@
         <v>106.6832</v>
       </c>
       <c r="I34" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="35">
@@ -1411,7 +1411,7 @@
         <v>106.6889</v>
       </c>
       <c r="I35" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="36">
@@ -1440,7 +1440,7 @@
         <v>106.6811</v>
       </c>
       <c r="I36" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="37">
@@ -1469,7 +1469,7 @@
         <v>106.705</v>
       </c>
       <c r="I37" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="38">
@@ -1498,7 +1498,7 @@
         <v>106.7052</v>
       </c>
       <c r="I38" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="39">
@@ -1527,7 +1527,7 @@
         <v>106.712</v>
       </c>
       <c r="I39" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="40">
@@ -1556,7 +1556,7 @@
         <v>106.638</v>
       </c>
       <c r="I40" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="41">
@@ -1585,7 +1585,7 @@
         <v>106.642</v>
       </c>
       <c r="I41" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="42">
@@ -1614,7 +1614,7 @@
         <v>106.6411</v>
       </c>
       <c r="I42" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="43">
@@ -1643,7 +1643,7 @@
         <v>106.6803</v>
       </c>
       <c r="I43" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="44">
@@ -1672,7 +1672,7 @@
         <v>106.653</v>
       </c>
       <c r="I44" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="45">
@@ -1701,7 +1701,7 @@
         <v>106.772</v>
       </c>
       <c r="I45" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="46">
@@ -1730,7 +1730,7 @@
         <v>106.7601</v>
       </c>
       <c r="I46" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="47">
@@ -1759,7 +1759,7 @@
         <v>106.7221</v>
       </c>
       <c r="I47" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="48">
@@ -1788,7 +1788,7 @@
         <v>106.7199</v>
       </c>
       <c r="I48" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="49">
@@ -1817,7 +1817,7 @@
         <v>106.702</v>
       </c>
       <c r="I49" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="50">
@@ -1846,7 +1846,7 @@
         <v>106.605</v>
       </c>
       <c r="I50" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="51">
@@ -1875,7 +1875,7 @@
         <v>106.6</v>
       </c>
       <c r="I51" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="52">
@@ -1904,7 +1904,7 @@
         <v>106.7033</v>
       </c>
       <c r="I52" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="53">
@@ -1933,7 +1933,7 @@
         <v>106.7071</v>
       </c>
       <c r="I53" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="54">
@@ -1962,7 +1962,7 @@
         <v>106.6981</v>
       </c>
       <c r="I54" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="55">
@@ -1991,7 +1991,7 @@
         <v>106.7009</v>
       </c>
       <c r="I55" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="56">
@@ -2020,7 +2020,7 @@
         <v>106.6961</v>
       </c>
       <c r="I56" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="57">
@@ -2049,7 +2049,7 @@
         <v>106.7012</v>
       </c>
       <c r="I57" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="58">
@@ -2078,7 +2078,7 @@
         <v>106.63</v>
       </c>
       <c r="I58" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="59">
@@ -2107,7 +2107,7 @@
         <v>106.6892</v>
       </c>
       <c r="I59" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="60">
@@ -2136,7 +2136,7 @@
         <v>106.6878</v>
       </c>
       <c r="I60" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="61">
@@ -2165,7 +2165,7 @@
         <v>106.693</v>
       </c>
       <c r="I61" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="62">
@@ -2194,7 +2194,7 @@
         <v>106.7052</v>
       </c>
       <c r="I62" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="63">
@@ -2223,7 +2223,7 @@
         <v>106.705</v>
       </c>
       <c r="I63" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
       </c>
     </row>
     <row r="64">
@@ -2252,12 +2252,41 @@
         <v>106.7018</v>
       </c>
       <c r="I64" t="str">
-        <v>2026-05-08T18:17:00.349Z</v>
+        <v>2026-05-09T04:27:53.251Z</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>e0b99ce7-906b-4dd8-88a6-9afed6432134</v>
+      </c>
+      <c r="B65" t="str">
+        <v>0368980079</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Home</v>
+      </c>
+      <c r="D65" t="str">
+        <v>354 Lý Thường Kiệt</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Q10</v>
+      </c>
+      <c r="F65" t="b">
+        <v>1</v>
+      </c>
+      <c r="G65">
+        <v>10.775595647737902</v>
+      </c>
+      <c r="H65">
+        <v>106.65752279721085</v>
+      </c>
+      <c r="I65" t="str">
+        <v>2026-05-09T04:30:55.379Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I65"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>